<commit_message>
feat: implement POS bargaining, real-time Khata ledger, delete orders with stock restoration, print receipt UX fixes, and supplier excel import
</commit_message>
<xml_diff>
--- a/public/assets/templates/supplier_import_template.xlsx
+++ b/public/assets/templates/supplier_import_template.xlsx
@@ -23,16 +23,16 @@
     <t>Phone</t>
   </si>
   <si>
-    <t>Email</t>
+    <t>Email (Optional)</t>
   </si>
   <si>
     <t>Address</t>
   </si>
   <si>
-    <t>Type</t>
-  </si>
-  <si>
-    <t>Shop Name</t>
+    <t>Type (Optional)</t>
+  </si>
+  <si>
+    <t>Shop Name (Optional)</t>
   </si>
   <si>
     <t>Total Bill</t>

</xml_diff>